<commit_message>
Fix アーカイブ送付 formula to reference new 開始時間 column
Old formula used C (時間 "10:00〜11:00" concat) which broke after C
became 日程短. New formula uses D (開始時間) directly:
=IF(IFERROR(TIMEVALUE(D_n),D_n)>TIME(13,0,0),B_n+1,B_n) — evening
events archive next day, morning/afternoon events archive same day.
IFERROR wrap lets it work whether D holds text "10:00" or a Time value.
動画配信 rows keep "-" (no archive mail).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019MpwpoXeU7u2s8oySrLx9o
</commit_message>
<xml_diff>
--- a/scratchpad/ShineALight_20ki_v3.xlsx
+++ b/scratchpad/ShineALight_20ki_v3.xlsx
@@ -29278,7 +29278,7 @@
         <v/>
       </c>
       <c r="L2" s="12">
-        <f>IF(TIMEVALUE(LEFT(C2, FIND("〜", C2&amp;"〜")-1)) &gt; TIME(13, 0, 0), B2+1, B2)</f>
+        <f>IF(IFERROR(TIMEVALUE(D2),D2)&gt;TIME(13,0,0),B2+1,B2)</f>
         <v/>
       </c>
       <c r="M2" s="15" t="inlineStr">
@@ -29428,7 +29428,7 @@
         <v/>
       </c>
       <c r="L4" s="12">
-        <f>IF(TIMEVALUE(LEFT(C4, FIND("〜", C4&amp;"〜")-1)) &gt; TIME(13, 0, 0), B4+1, B4)</f>
+        <f>IF(IFERROR(TIMEVALUE(D4),D4)&gt;TIME(13,0,0),B4+1,B4)</f>
         <v/>
       </c>
       <c r="M4" s="15" t="inlineStr">
@@ -29498,7 +29498,7 @@
         <v/>
       </c>
       <c r="L5" s="12">
-        <f>IF(TIMEVALUE(LEFT(C5, FIND("〜", C5&amp;"〜")-1)) &gt; TIME(13, 0, 0), B5+1, B5)</f>
+        <f>IF(IFERROR(TIMEVALUE(D5),D5)&gt;TIME(13,0,0),B5+1,B5)</f>
         <v/>
       </c>
       <c r="M5" s="15" t="inlineStr">
@@ -29570,7 +29570,7 @@
         <v/>
       </c>
       <c r="L6" s="12">
-        <f>IF(TIMEVALUE(LEFT(C6, FIND("〜", C6&amp;"〜")-1)) &gt; TIME(13, 0, 0), B6+1, B6)</f>
+        <f>IF(IFERROR(TIMEVALUE(D6),D6)&gt;TIME(13,0,0),B6+1,B6)</f>
         <v/>
       </c>
       <c r="M6" s="15" t="inlineStr">
@@ -29640,7 +29640,7 @@
         <v/>
       </c>
       <c r="L7" s="12">
-        <f>IF(TIMEVALUE(LEFT(C7, FIND("〜", C7&amp;"〜")-1)) &gt; TIME(13, 0, 0), B7+1, B7)</f>
+        <f>IF(IFERROR(TIMEVALUE(D7),D7)&gt;TIME(13,0,0),B7+1,B7)</f>
         <v/>
       </c>
       <c r="M7" s="15" t="inlineStr">
@@ -29782,7 +29782,7 @@
         <v/>
       </c>
       <c r="L9" s="12">
-        <f>IF(TIMEVALUE(LEFT(C9, FIND("〜", C9&amp;"〜")-1)) &gt; TIME(13, 0, 0), B9+1, B9)</f>
+        <f>IF(IFERROR(TIMEVALUE(D9),D9)&gt;TIME(13,0,0),B9+1,B9)</f>
         <v/>
       </c>
       <c r="M9" s="15" t="inlineStr">
@@ -29854,7 +29854,7 @@
         <v/>
       </c>
       <c r="L10" s="12">
-        <f>IF(TIMEVALUE(LEFT(C10, FIND("〜", C10&amp;"〜")-1)) &gt; TIME(13, 0, 0), B10+1, B10)</f>
+        <f>IF(IFERROR(TIMEVALUE(D10),D10)&gt;TIME(13,0,0),B10+1,B10)</f>
         <v/>
       </c>
       <c r="M10" s="15" t="inlineStr">
@@ -29924,7 +29924,7 @@
         <v/>
       </c>
       <c r="L11" s="12">
-        <f>IF(TIMEVALUE(LEFT(C11, FIND("〜", C11&amp;"〜")-1)) &gt; TIME(13, 0, 0), B11+1, B11)</f>
+        <f>IF(IFERROR(TIMEVALUE(D11),D11)&gt;TIME(13,0,0),B11+1,B11)</f>
         <v/>
       </c>
       <c r="M11" s="15" t="inlineStr">
@@ -30066,7 +30066,7 @@
         <v/>
       </c>
       <c r="L13" s="12">
-        <f>IF(TIMEVALUE(LEFT(C13, FIND("〜", C13&amp;"〜")-1)) &gt; TIME(13, 0, 0), B13+1, B13)</f>
+        <f>IF(IFERROR(TIMEVALUE(D13),D13)&gt;TIME(13,0,0),B13+1,B13)</f>
         <v/>
       </c>
       <c r="M13" s="15" t="inlineStr">
@@ -30136,7 +30136,7 @@
         <v/>
       </c>
       <c r="L14" s="12">
-        <f>IF(TIMEVALUE(LEFT(C14, FIND("〜", C14&amp;"〜")-1)) &gt; TIME(13, 0, 0), B14+1, B14)</f>
+        <f>IF(IFERROR(TIMEVALUE(D14),D14)&gt;TIME(13,0,0),B14+1,B14)</f>
         <v/>
       </c>
       <c r="M14" s="15" t="inlineStr">
@@ -30208,7 +30208,7 @@
         <v/>
       </c>
       <c r="L15" s="12">
-        <f>IF(TIMEVALUE(LEFT(C15, FIND("〜", C15&amp;"〜")-1)) &gt; TIME(13, 0, 0), B15+1, B15)</f>
+        <f>IF(IFERROR(TIMEVALUE(D15),D15)&gt;TIME(13,0,0),B15+1,B15)</f>
         <v/>
       </c>
       <c r="M15" s="15" t="inlineStr">
@@ -30278,7 +30278,7 @@
         <v/>
       </c>
       <c r="L16" s="12">
-        <f>IF(TIMEVALUE(LEFT(C16, FIND("〜", C16&amp;"〜")-1)) &gt; TIME(13, 0, 0), B16+1, B16)</f>
+        <f>IF(IFERROR(TIMEVALUE(D16),D16)&gt;TIME(13,0,0),B16+1,B16)</f>
         <v/>
       </c>
       <c r="M16" s="15" t="inlineStr">
@@ -30418,7 +30418,7 @@
         <v/>
       </c>
       <c r="L18" s="12">
-        <f>IF(TIMEVALUE(LEFT(C18, FIND("〜", C18&amp;"〜")-1)) &gt; TIME(13, 0, 0), B18+1, B18)</f>
+        <f>IF(IFERROR(TIMEVALUE(D18),D18)&gt;TIME(13,0,0),B18+1,B18)</f>
         <v/>
       </c>
       <c r="M18" s="15" t="inlineStr">
@@ -30490,7 +30490,7 @@
         <v/>
       </c>
       <c r="L19" s="12">
-        <f>IF(TIMEVALUE(LEFT(C19, FIND("〜", C19&amp;"〜")-1)) &gt; TIME(13, 0, 0), B19+1, B19)</f>
+        <f>IF(IFERROR(TIMEVALUE(D19),D19)&gt;TIME(13,0,0),B19+1,B19)</f>
         <v/>
       </c>
       <c r="M19" s="15" t="inlineStr">
@@ -30560,7 +30560,7 @@
         <v/>
       </c>
       <c r="L20" s="12">
-        <f>IF(TIMEVALUE(LEFT(C20, FIND("〜", C20&amp;"〜")-1)) &gt; TIME(13, 0, 0), B20+1, B20)</f>
+        <f>IF(IFERROR(TIMEVALUE(D20),D20)&gt;TIME(13,0,0),B20+1,B20)</f>
         <v/>
       </c>
       <c r="M20" s="15" t="inlineStr">
@@ -30632,7 +30632,7 @@
         <v/>
       </c>
       <c r="L21" s="12">
-        <f>IF(TIMEVALUE(LEFT(C21, FIND("〜", C21&amp;"〜")-1)) &gt; TIME(13, 0, 0), B21+1, B21)</f>
+        <f>IF(IFERROR(TIMEVALUE(D21),D21)&gt;TIME(13,0,0),B21+1,B21)</f>
         <v/>
       </c>
       <c r="M21" s="15" t="inlineStr">
@@ -30702,7 +30702,7 @@
         <v/>
       </c>
       <c r="L22" s="12">
-        <f>IF(TIMEVALUE(LEFT(C22, FIND("〜", C22&amp;"〜")-1)) &gt; TIME(13, 0, 0), B22+1, B22)</f>
+        <f>IF(IFERROR(TIMEVALUE(D22),D22)&gt;TIME(13,0,0),B22+1,B22)</f>
         <v/>
       </c>
       <c r="M22" s="15" t="inlineStr">
@@ -30844,7 +30844,7 @@
         <v/>
       </c>
       <c r="L24" s="12">
-        <f>IF(TIMEVALUE(LEFT(C24, FIND("〜", C24&amp;"〜")-1)) &gt; TIME(13, 0, 0), B24+1, B24)</f>
+        <f>IF(IFERROR(TIMEVALUE(D24),D24)&gt;TIME(13,0,0),B24+1,B24)</f>
         <v/>
       </c>
       <c r="M24" s="15" t="inlineStr">
@@ -30916,7 +30916,7 @@
         <v/>
       </c>
       <c r="L25" s="12">
-        <f>IF(TIMEVALUE(LEFT(C25, FIND("〜", C25&amp;"〜")-1)) &gt; TIME(13, 0, 0), B25+1, B25)</f>
+        <f>IF(IFERROR(TIMEVALUE(D25),D25)&gt;TIME(13,0,0),B25+1,B25)</f>
         <v/>
       </c>
       <c r="M25" s="15" t="inlineStr">
@@ -30986,7 +30986,7 @@
         <v/>
       </c>
       <c r="L26" s="12">
-        <f>IF(TIMEVALUE(LEFT(C26, FIND("〜", C26&amp;"〜")-1)) &gt; TIME(13, 0, 0), B26+1, B26)</f>
+        <f>IF(IFERROR(TIMEVALUE(D26),D26)&gt;TIME(13,0,0),B26+1,B26)</f>
         <v/>
       </c>
       <c r="M26" s="15" t="inlineStr">
@@ -31056,7 +31056,7 @@
         <v/>
       </c>
       <c r="L27" s="12">
-        <f>IF(TIMEVALUE(LEFT(C27, FIND("〜", C27&amp;"〜")-1)) &gt; TIME(13, 0, 0), B27+1, B27)</f>
+        <f>IF(IFERROR(TIMEVALUE(D27),D27)&gt;TIME(13,0,0),B27+1,B27)</f>
         <v/>
       </c>
       <c r="M27" s="15" t="inlineStr">
@@ -31196,7 +31196,7 @@
         <v/>
       </c>
       <c r="L29" s="12">
-        <f>IF(TIMEVALUE(LEFT(C29, FIND("〜", C29&amp;"〜")-1)) &gt; TIME(13, 0, 0), B29+1, B29)</f>
+        <f>IF(IFERROR(TIMEVALUE(D29),D29)&gt;TIME(13,0,0),B29+1,B29)</f>
         <v/>
       </c>
       <c r="M29" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Drop ID column from スケジュール
The ID column (E001..E029) was reserved for future extensions but no
current code path references it. Removing it shrinks the sheet from
17 to 16 columns. GAS side: COL constants renumbered, event.id and
{{ID}} variable dropped.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019MpwpoXeU7u2s8oySrLx9o
</commit_message>
<xml_diff>
--- a/scratchpad/ShineALight_20ki_v3.xlsx
+++ b/scratchpad/ShineALight_20ki_v3.xlsx
@@ -275,7 +275,7 @@
         <t>=IF(B2="","",TEXT(B2,"M/d（aaa）")) で自動計算</t>
       </text>
     </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
+    <comment ref="M1" authorId="0" shapeId="0">
       <text>
         <t>選択肢：若菜グルコン共通 / 若菜マンデー共通 / 個別 / 未定(サポート講師待ち) / Zoomなし</t>
       </text>
@@ -29118,7 +29118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q29"/>
+  <dimension ref="A1:P29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -29133,11 +29133,10 @@
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="40" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -29203,25 +29202,20 @@
       </c>
       <c r="M1" s="13" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>Zoomソース</t>
         </is>
       </c>
       <c r="N1" s="13" t="inlineStr">
         <is>
-          <t>Zoomソース</t>
+          <t>Zoomリンク</t>
         </is>
       </c>
       <c r="O1" s="13" t="inlineStr">
         <is>
-          <t>Zoomリンク</t>
+          <t>ミーティングID</t>
         </is>
       </c>
       <c r="P1" s="13" t="inlineStr">
-        <is>
-          <t>ミーティングID</t>
-        </is>
-      </c>
-      <c r="Q1" s="13" t="inlineStr">
         <is>
           <t>ステータス</t>
         </is>
@@ -29281,27 +29275,22 @@
         <f>IF(IFERROR(TIMEVALUE(D2),D2)&gt;TIME(13,0,0),B2+1,B2)</f>
         <v/>
       </c>
-      <c r="M2" s="15" t="inlineStr">
-        <is>
-          <t>E001</t>
-        </is>
-      </c>
-      <c r="N2" s="10" t="inlineStr">
+      <c r="M2" s="10" t="inlineStr">
         <is>
           <t>個別</t>
         </is>
       </c>
+      <c r="N2" s="12" t="inlineStr">
+        <is>
+          <t>https://us02web.zoom.us/j/82603439180</t>
+        </is>
+      </c>
       <c r="O2" s="12" t="inlineStr">
         <is>
-          <t>https://us02web.zoom.us/j/82603439180</t>
+          <t>826 0343 9180</t>
         </is>
       </c>
       <c r="P2" s="12" t="inlineStr">
-        <is>
-          <t>826 0343 9180</t>
-        </is>
-      </c>
-      <c r="Q2" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -29359,19 +29348,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M3" s="15" t="inlineStr">
-        <is>
-          <t>E002</t>
-        </is>
-      </c>
-      <c r="N3" s="10" t="inlineStr">
+      <c r="M3" s="10" t="inlineStr">
         <is>
           <t>Zoomなし</t>
         </is>
       </c>
+      <c r="N3" s="12" t="n"/>
       <c r="O3" s="12" t="n"/>
-      <c r="P3" s="12" t="n"/>
-      <c r="Q3" s="12" t="inlineStr">
+      <c r="P3" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -29431,19 +29415,14 @@
         <f>IF(IFERROR(TIMEVALUE(D4),D4)&gt;TIME(13,0,0),B4+1,B4)</f>
         <v/>
       </c>
-      <c r="M4" s="15" t="inlineStr">
-        <is>
-          <t>E003</t>
-        </is>
-      </c>
-      <c r="N4" s="10" t="inlineStr">
+      <c r="M4" s="10" t="inlineStr">
         <is>
           <t>未定(サポート講師待ち)</t>
         </is>
       </c>
+      <c r="N4" s="12" t="n"/>
       <c r="O4" s="12" t="n"/>
-      <c r="P4" s="12" t="n"/>
-      <c r="Q4" s="12" t="inlineStr">
+      <c r="P4" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -29501,19 +29480,14 @@
         <f>IF(IFERROR(TIMEVALUE(D5),D5)&gt;TIME(13,0,0),B5+1,B5)</f>
         <v/>
       </c>
-      <c r="M5" s="15" t="inlineStr">
-        <is>
-          <t>E004</t>
-        </is>
-      </c>
-      <c r="N5" s="10" t="inlineStr">
+      <c r="M5" s="10" t="inlineStr">
         <is>
           <t>未定(サポート講師待ち)</t>
         </is>
       </c>
+      <c r="N5" s="12" t="n"/>
       <c r="O5" s="12" t="n"/>
-      <c r="P5" s="12" t="n"/>
-      <c r="Q5" s="12" t="inlineStr">
+      <c r="P5" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -29573,19 +29547,14 @@
         <f>IF(IFERROR(TIMEVALUE(D6),D6)&gt;TIME(13,0,0),B6+1,B6)</f>
         <v/>
       </c>
-      <c r="M6" s="15" t="inlineStr">
-        <is>
-          <t>E005</t>
-        </is>
-      </c>
-      <c r="N6" s="10" t="inlineStr">
+      <c r="M6" s="10" t="inlineStr">
         <is>
           <t>若菜マンデー共通</t>
         </is>
       </c>
+      <c r="N6" s="12" t="n"/>
       <c r="O6" s="12" t="n"/>
-      <c r="P6" s="12" t="n"/>
-      <c r="Q6" s="12" t="inlineStr">
+      <c r="P6" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -29643,19 +29612,14 @@
         <f>IF(IFERROR(TIMEVALUE(D7),D7)&gt;TIME(13,0,0),B7+1,B7)</f>
         <v/>
       </c>
-      <c r="M7" s="15" t="inlineStr">
-        <is>
-          <t>E006</t>
-        </is>
-      </c>
-      <c r="N7" s="10" t="inlineStr">
+      <c r="M7" s="10" t="inlineStr">
         <is>
           <t>若菜グルコン共通</t>
         </is>
       </c>
+      <c r="N7" s="12" t="n"/>
       <c r="O7" s="12" t="n"/>
-      <c r="P7" s="12" t="n"/>
-      <c r="Q7" s="12" t="inlineStr">
+      <c r="P7" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -29713,19 +29677,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M8" s="15" t="inlineStr">
-        <is>
-          <t>E007</t>
-        </is>
-      </c>
-      <c r="N8" s="10" t="inlineStr">
+      <c r="M8" s="10" t="inlineStr">
         <is>
           <t>Zoomなし</t>
         </is>
       </c>
+      <c r="N8" s="12" t="n"/>
       <c r="O8" s="12" t="n"/>
-      <c r="P8" s="12" t="n"/>
-      <c r="Q8" s="12" t="inlineStr">
+      <c r="P8" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -29785,19 +29744,14 @@
         <f>IF(IFERROR(TIMEVALUE(D9),D9)&gt;TIME(13,0,0),B9+1,B9)</f>
         <v/>
       </c>
-      <c r="M9" s="15" t="inlineStr">
-        <is>
-          <t>E008</t>
-        </is>
-      </c>
-      <c r="N9" s="10" t="inlineStr">
+      <c r="M9" s="10" t="inlineStr">
         <is>
           <t>未定(サポート講師待ち)</t>
         </is>
       </c>
+      <c r="N9" s="12" t="n"/>
       <c r="O9" s="12" t="n"/>
-      <c r="P9" s="12" t="n"/>
-      <c r="Q9" s="12" t="inlineStr">
+      <c r="P9" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -29857,19 +29811,14 @@
         <f>IF(IFERROR(TIMEVALUE(D10),D10)&gt;TIME(13,0,0),B10+1,B10)</f>
         <v/>
       </c>
-      <c r="M10" s="15" t="inlineStr">
-        <is>
-          <t>E009</t>
-        </is>
-      </c>
-      <c r="N10" s="10" t="inlineStr">
+      <c r="M10" s="10" t="inlineStr">
         <is>
           <t>若菜マンデー共通</t>
         </is>
       </c>
+      <c r="N10" s="12" t="n"/>
       <c r="O10" s="12" t="n"/>
-      <c r="P10" s="12" t="n"/>
-      <c r="Q10" s="12" t="inlineStr">
+      <c r="P10" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -29927,19 +29876,14 @@
         <f>IF(IFERROR(TIMEVALUE(D11),D11)&gt;TIME(13,0,0),B11+1,B11)</f>
         <v/>
       </c>
-      <c r="M11" s="15" t="inlineStr">
-        <is>
-          <t>E010</t>
-        </is>
-      </c>
-      <c r="N11" s="10" t="inlineStr">
+      <c r="M11" s="10" t="inlineStr">
         <is>
           <t>若菜グルコン共通</t>
         </is>
       </c>
+      <c r="N11" s="12" t="n"/>
       <c r="O11" s="12" t="n"/>
-      <c r="P11" s="12" t="n"/>
-      <c r="Q11" s="12" t="inlineStr">
+      <c r="P11" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -29997,19 +29941,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M12" s="15" t="inlineStr">
-        <is>
-          <t>E011</t>
-        </is>
-      </c>
-      <c r="N12" s="10" t="inlineStr">
+      <c r="M12" s="10" t="inlineStr">
         <is>
           <t>Zoomなし</t>
         </is>
       </c>
+      <c r="N12" s="12" t="n"/>
       <c r="O12" s="12" t="n"/>
-      <c r="P12" s="12" t="n"/>
-      <c r="Q12" s="12" t="inlineStr">
+      <c r="P12" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -30069,19 +30008,14 @@
         <f>IF(IFERROR(TIMEVALUE(D13),D13)&gt;TIME(13,0,0),B13+1,B13)</f>
         <v/>
       </c>
-      <c r="M13" s="15" t="inlineStr">
-        <is>
-          <t>E012</t>
-        </is>
-      </c>
-      <c r="N13" s="10" t="inlineStr">
+      <c r="M13" s="10" t="inlineStr">
         <is>
           <t>未定(サポート講師待ち)</t>
         </is>
       </c>
+      <c r="N13" s="12" t="n"/>
       <c r="O13" s="12" t="n"/>
-      <c r="P13" s="12" t="n"/>
-      <c r="Q13" s="12" t="inlineStr">
+      <c r="P13" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -30139,19 +30073,14 @@
         <f>IF(IFERROR(TIMEVALUE(D14),D14)&gt;TIME(13,0,0),B14+1,B14)</f>
         <v/>
       </c>
-      <c r="M14" s="15" t="inlineStr">
-        <is>
-          <t>E013</t>
-        </is>
-      </c>
-      <c r="N14" s="10" t="inlineStr">
+      <c r="M14" s="10" t="inlineStr">
         <is>
           <t>未定(サポート講師待ち)</t>
         </is>
       </c>
+      <c r="N14" s="12" t="n"/>
       <c r="O14" s="12" t="n"/>
-      <c r="P14" s="12" t="n"/>
-      <c r="Q14" s="12" t="inlineStr">
+      <c r="P14" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -30211,19 +30140,14 @@
         <f>IF(IFERROR(TIMEVALUE(D15),D15)&gt;TIME(13,0,0),B15+1,B15)</f>
         <v/>
       </c>
-      <c r="M15" s="15" t="inlineStr">
-        <is>
-          <t>E014</t>
-        </is>
-      </c>
-      <c r="N15" s="10" t="inlineStr">
+      <c r="M15" s="10" t="inlineStr">
         <is>
           <t>若菜マンデー共通</t>
         </is>
       </c>
+      <c r="N15" s="12" t="n"/>
       <c r="O15" s="12" t="n"/>
-      <c r="P15" s="12" t="n"/>
-      <c r="Q15" s="12" t="inlineStr">
+      <c r="P15" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -30281,19 +30205,14 @@
         <f>IF(IFERROR(TIMEVALUE(D16),D16)&gt;TIME(13,0,0),B16+1,B16)</f>
         <v/>
       </c>
-      <c r="M16" s="15" t="inlineStr">
-        <is>
-          <t>E015</t>
-        </is>
-      </c>
-      <c r="N16" s="10" t="inlineStr">
+      <c r="M16" s="10" t="inlineStr">
         <is>
           <t>若菜グルコン共通</t>
         </is>
       </c>
+      <c r="N16" s="12" t="n"/>
       <c r="O16" s="12" t="n"/>
-      <c r="P16" s="12" t="n"/>
-      <c r="Q16" s="12" t="inlineStr">
+      <c r="P16" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -30351,19 +30270,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M17" s="15" t="inlineStr">
-        <is>
-          <t>E016</t>
-        </is>
-      </c>
-      <c r="N17" s="10" t="inlineStr">
+      <c r="M17" s="10" t="inlineStr">
         <is>
           <t>Zoomなし</t>
         </is>
       </c>
+      <c r="N17" s="12" t="n"/>
       <c r="O17" s="12" t="n"/>
-      <c r="P17" s="12" t="n"/>
-      <c r="Q17" s="12" t="inlineStr">
+      <c r="P17" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -30421,19 +30335,14 @@
         <f>IF(IFERROR(TIMEVALUE(D18),D18)&gt;TIME(13,0,0),B18+1,B18)</f>
         <v/>
       </c>
-      <c r="M18" s="15" t="inlineStr">
-        <is>
-          <t>E017</t>
-        </is>
-      </c>
-      <c r="N18" s="10" t="inlineStr">
+      <c r="M18" s="10" t="inlineStr">
         <is>
           <t>個別</t>
         </is>
       </c>
+      <c r="N18" s="12" t="n"/>
       <c r="O18" s="12" t="n"/>
-      <c r="P18" s="12" t="n"/>
-      <c r="Q18" s="12" t="inlineStr">
+      <c r="P18" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -30493,19 +30402,14 @@
         <f>IF(IFERROR(TIMEVALUE(D19),D19)&gt;TIME(13,0,0),B19+1,B19)</f>
         <v/>
       </c>
-      <c r="M19" s="15" t="inlineStr">
-        <is>
-          <t>E018</t>
-        </is>
-      </c>
-      <c r="N19" s="10" t="inlineStr">
+      <c r="M19" s="10" t="inlineStr">
         <is>
           <t>未定(サポート講師待ち)</t>
         </is>
       </c>
+      <c r="N19" s="12" t="n"/>
       <c r="O19" s="12" t="n"/>
-      <c r="P19" s="12" t="n"/>
-      <c r="Q19" s="12" t="inlineStr">
+      <c r="P19" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -30563,19 +30467,14 @@
         <f>IF(IFERROR(TIMEVALUE(D20),D20)&gt;TIME(13,0,0),B20+1,B20)</f>
         <v/>
       </c>
-      <c r="M20" s="15" t="inlineStr">
-        <is>
-          <t>E019</t>
-        </is>
-      </c>
-      <c r="N20" s="10" t="inlineStr">
+      <c r="M20" s="10" t="inlineStr">
         <is>
           <t>未定(サポート講師待ち)</t>
         </is>
       </c>
+      <c r="N20" s="12" t="n"/>
       <c r="O20" s="12" t="n"/>
-      <c r="P20" s="12" t="n"/>
-      <c r="Q20" s="12" t="inlineStr">
+      <c r="P20" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -30635,19 +30534,14 @@
         <f>IF(IFERROR(TIMEVALUE(D21),D21)&gt;TIME(13,0,0),B21+1,B21)</f>
         <v/>
       </c>
-      <c r="M21" s="15" t="inlineStr">
-        <is>
-          <t>E020</t>
-        </is>
-      </c>
-      <c r="N21" s="10" t="inlineStr">
+      <c r="M21" s="10" t="inlineStr">
         <is>
           <t>若菜マンデー共通</t>
         </is>
       </c>
+      <c r="N21" s="12" t="n"/>
       <c r="O21" s="12" t="n"/>
-      <c r="P21" s="12" t="n"/>
-      <c r="Q21" s="12" t="inlineStr">
+      <c r="P21" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -30705,19 +30599,14 @@
         <f>IF(IFERROR(TIMEVALUE(D22),D22)&gt;TIME(13,0,0),B22+1,B22)</f>
         <v/>
       </c>
-      <c r="M22" s="15" t="inlineStr">
-        <is>
-          <t>E021</t>
-        </is>
-      </c>
-      <c r="N22" s="10" t="inlineStr">
+      <c r="M22" s="10" t="inlineStr">
         <is>
           <t>若菜グルコン共通</t>
         </is>
       </c>
+      <c r="N22" s="12" t="n"/>
       <c r="O22" s="12" t="n"/>
-      <c r="P22" s="12" t="n"/>
-      <c r="Q22" s="12" t="inlineStr">
+      <c r="P22" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -30775,19 +30664,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M23" s="15" t="inlineStr">
-        <is>
-          <t>E022</t>
-        </is>
-      </c>
-      <c r="N23" s="10" t="inlineStr">
+      <c r="M23" s="10" t="inlineStr">
         <is>
           <t>Zoomなし</t>
         </is>
       </c>
+      <c r="N23" s="12" t="n"/>
       <c r="O23" s="12" t="n"/>
-      <c r="P23" s="12" t="n"/>
-      <c r="Q23" s="12" t="inlineStr">
+      <c r="P23" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -30847,19 +30731,14 @@
         <f>IF(IFERROR(TIMEVALUE(D24),D24)&gt;TIME(13,0,0),B24+1,B24)</f>
         <v/>
       </c>
-      <c r="M24" s="15" t="inlineStr">
-        <is>
-          <t>E023</t>
-        </is>
-      </c>
-      <c r="N24" s="10" t="inlineStr">
+      <c r="M24" s="10" t="inlineStr">
         <is>
           <t>未定(サポート講師待ち)</t>
         </is>
       </c>
+      <c r="N24" s="12" t="n"/>
       <c r="O24" s="12" t="n"/>
-      <c r="P24" s="12" t="n"/>
-      <c r="Q24" s="12" t="inlineStr">
+      <c r="P24" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -30919,19 +30798,14 @@
         <f>IF(IFERROR(TIMEVALUE(D25),D25)&gt;TIME(13,0,0),B25+1,B25)</f>
         <v/>
       </c>
-      <c r="M25" s="15" t="inlineStr">
-        <is>
-          <t>E024</t>
-        </is>
-      </c>
-      <c r="N25" s="10" t="inlineStr">
+      <c r="M25" s="10" t="inlineStr">
         <is>
           <t>若菜マンデー共通</t>
         </is>
       </c>
+      <c r="N25" s="12" t="n"/>
       <c r="O25" s="12" t="n"/>
-      <c r="P25" s="12" t="n"/>
-      <c r="Q25" s="12" t="inlineStr">
+      <c r="P25" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -30989,19 +30863,14 @@
         <f>IF(IFERROR(TIMEVALUE(D26),D26)&gt;TIME(13,0,0),B26+1,B26)</f>
         <v/>
       </c>
-      <c r="M26" s="15" t="inlineStr">
-        <is>
-          <t>E025</t>
-        </is>
-      </c>
-      <c r="N26" s="10" t="inlineStr">
+      <c r="M26" s="10" t="inlineStr">
         <is>
           <t>若菜グルコン共通</t>
         </is>
       </c>
+      <c r="N26" s="12" t="n"/>
       <c r="O26" s="12" t="n"/>
-      <c r="P26" s="12" t="n"/>
-      <c r="Q26" s="12" t="inlineStr">
+      <c r="P26" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -31059,19 +30928,14 @@
         <f>IF(IFERROR(TIMEVALUE(D27),D27)&gt;TIME(13,0,0),B27+1,B27)</f>
         <v/>
       </c>
-      <c r="M27" s="15" t="inlineStr">
-        <is>
-          <t>E026</t>
-        </is>
-      </c>
-      <c r="N27" s="10" t="inlineStr">
+      <c r="M27" s="10" t="inlineStr">
         <is>
           <t>未定(サポート講師待ち)</t>
         </is>
       </c>
+      <c r="N27" s="12" t="n"/>
       <c r="O27" s="12" t="n"/>
-      <c r="P27" s="12" t="n"/>
-      <c r="Q27" s="12" t="inlineStr">
+      <c r="P27" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -31129,19 +30993,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M28" s="15" t="inlineStr">
-        <is>
-          <t>E027</t>
-        </is>
-      </c>
-      <c r="N28" s="10" t="inlineStr">
+      <c r="M28" s="10" t="inlineStr">
         <is>
           <t>Zoomなし</t>
         </is>
       </c>
+      <c r="N28" s="12" t="n"/>
       <c r="O28" s="12" t="n"/>
-      <c r="P28" s="12" t="n"/>
-      <c r="Q28" s="12" t="inlineStr">
+      <c r="P28" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>
@@ -31199,19 +31058,14 @@
         <f>IF(IFERROR(TIMEVALUE(D29),D29)&gt;TIME(13,0,0),B29+1,B29)</f>
         <v/>
       </c>
-      <c r="M29" s="15" t="inlineStr">
-        <is>
-          <t>E028</t>
-        </is>
-      </c>
-      <c r="N29" s="10" t="inlineStr">
+      <c r="M29" s="10" t="inlineStr">
         <is>
           <t>若菜グルコン共通</t>
         </is>
       </c>
+      <c r="N29" s="12" t="n"/>
       <c r="O29" s="12" t="n"/>
-      <c r="P29" s="12" t="n"/>
-      <c r="Q29" s="12" t="inlineStr">
+      <c r="P29" s="12" t="inlineStr">
         <is>
           <t>未実施</t>
         </is>

</xml_diff>